<commit_message>
blatt-hefte: RNB from a budget base, new Budsjettloep sheet
UiT RNB changes are not in the RNB proposition (sector totals only) but
in KD supplementary allocation letter no. 1 to state universities,
published on regjeringen.no ~5 weeks after the proposition. Map for
2024-2026 (Prop. 104/146/96 S, letters 25.06.2024, 02.07.2025,
25.06.2026; UiT +8 300, -907, +364) in the source map with paths R1-R7.

rnb-tillegg.json holds the per-year UiT change with components, url,
sha256 and date; bygg_base.py reads forslag and vedtatt for 2021-2026
from the hefter and writes budsjettbase.json. The workbook fills the
RNB cell for the year before from the base (override with --rnb),
gets a Budsjettloep sheet (forslag, vedtatt, RNB, vedtatt incl. RNB,
source) and an RNB source row in Kilder. 67 tests.
</commit_message>
<xml_diff>
--- a/skills/knowledge-management/blatt-hefte/assets/mal-rammeark.xlsx
+++ b/skills/knowledge-management/blatt-hefte/assets/mal-rammeark.xlsx
@@ -8,14 +8,18 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hovedtall" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hovedposter" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultat" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sektor" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Satser" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kilder" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_meta" sheetId="7" state="hidden" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budsjettløp" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hovedposter" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultat" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sektor" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Satser" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kilder" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_meta" sheetId="8" state="hidden" r:id="rId8"/>
   </sheets>
   <definedNames>
+    <definedName name="budsjettloep_merknad">'Budsjettløp'!$B$13</definedName>
+    <definedName name="budsjettloep_overskrift">'Budsjettløp'!$B$5</definedName>
+    <definedName name="budsjettloep_start">'Budsjettløp'!$B$6</definedName>
     <definedName name="hovedposter_kontroll">'Hovedposter'!$D$20</definedName>
     <definedName name="hovedposter_overskrift">'Hovedposter'!$B$5</definedName>
     <definedName name="hovedposter_rnb_forslag">'Hovedposter'!$C$24</definedName>
@@ -43,12 +47,13 @@
     <definedName name="kilder_budsjettaar">'Kilder'!$C$6</definedName>
     <definedName name="kilder_content_length">'Kilder'!$C$12</definedName>
     <definedName name="kilder_filnavn">'Kilder'!$C$10</definedName>
-    <definedName name="kilder_finn_dom">'Kilder'!$C$33</definedName>
+    <definedName name="kilder_finn_dom">'Kilder'!$C$34</definedName>
     <definedName name="kilder_hentet">'Kilder'!$C$13</definedName>
-    <definedName name="kilder_kjort">'Kilder'!$C$32</definedName>
-    <definedName name="kilder_kontroll_a">'Kilder'!$C$27</definedName>
-    <definedName name="kilder_kontroll_b">'Kilder'!$C$28</definedName>
-    <definedName name="kilder_kontroll_c">'Kilder'!$C$29</definedName>
+    <definedName name="kilder_kjort">'Kilder'!$C$33</definedName>
+    <definedName name="kilder_kontroll_a">'Kilder'!$C$28</definedName>
+    <definedName name="kilder_kontroll_b">'Kilder'!$C$29</definedName>
+    <definedName name="kilder_kontroll_c">'Kilder'!$C$30</definedName>
+    <definedName name="kilder_rnb">'Kilder'!$C$26</definedName>
     <definedName name="kilder_sha256">'Kilder'!$C$11</definedName>
     <definedName name="kilder_side_hovedtabell">'Kilder'!$C$17</definedName>
     <definedName name="kilder_side_institusjoner">'Kilder'!$C$23</definedName>
@@ -58,9 +63,9 @@
     <definedName name="kilder_side_satser">'Kilder'!$C$21</definedName>
     <definedName name="kilder_side_trykt">'Kilder'!$C$18</definedName>
     <definedName name="kilder_sider">'Kilder'!$C$14</definedName>
-    <definedName name="kilder_sitat">'Kilder'!$C$26</definedName>
-    <definedName name="kilder_skript">'Kilder'!$C$30</definedName>
-    <definedName name="kilder_skriptversjon">'Kilder'!$C$31</definedName>
+    <definedName name="kilder_sitat">'Kilder'!$C$27</definedName>
+    <definedName name="kilder_skript">'Kilder'!$C$31</definedName>
+    <definedName name="kilder_skriptversjon">'Kilder'!$C$32</definedName>
     <definedName name="kilder_tittel">'Kilder'!$C$8</definedName>
     <definedName name="kilder_url">'Kilder'!$C$9</definedName>
     <definedName name="kilder_utgave">'Kilder'!$C$7</definedName>
@@ -705,6 +710,136 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B2:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2.5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Budsjettløpet for UiT: forslag, vedtatt og revidert</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>NOK i hele tusen</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Budsjettår</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Forslag (blått hefte)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Vedtatt (etter Stortinget)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>RNB-tillegg</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Vedtatt inkl. RNB</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>RNB-kilde</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4">
+        <f>IF(OR(D6="",E6=""),"ikke oppgitt",D6+E6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="n"/>
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="4">
+        <f>IF(OR(D7="",E7=""),"ikke oppgitt",D7+E7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="4" t="n"/>
+      <c r="E8" s="4" t="n"/>
+      <c r="F8" s="4">
+        <f>IF(OR(D8="",E8=""),"ikke oppgitt",D8+E8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="4">
+        <f>IF(OR(D9="",E9=""),"ikke oppgitt",D9+E9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="4" t="n"/>
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="4">
+        <f>IF(OR(D10="",E10=""),"ikke oppgitt",D10+E10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="4" t="n"/>
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4">
+        <f>IF(OR(D11="",E11=""),"ikke oppgitt",D11+E11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>RNB-tillegget er UiTs endring på kap. 260 post 50 i KDs supplerende tildelingsbrev nr. 1 etter revidert nasjonalbudsjett (juni/juli). Proposisjonen har bare sektortall, og blått hefte har ingen RNB-utgave. Realvekst «med RNB» i Hovedtall bruker RNB-tillegget for året før som del av utgangspunktet.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -867,7 +1002,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -943,7 +1078,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1472,7 +1607,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1541,13 +1676,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C33"/>
+  <dimension ref="B2:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -1722,54 +1857,61 @@
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>Prissats-sitat</t>
+          <t>RNB-tillegg brukt i Hovedtall (året før, kilde)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" t="inlineStr">
         <is>
-          <t>Kontroll A (alle rader summerer)</t>
+          <t>Prissats-sitat</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>Kontroll B (bånd mot overskrifter)</t>
+          <t>Kontroll A (alle rader summerer)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>Kontroll C (kryss mot forrige hefte)</t>
+          <t>Kontroll B (bånd mot overskrifter)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>Skript</t>
+          <t>Kontroll C (kryss mot forrige hefte)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
-          <t>Skriptversjon</t>
+          <t>Skript</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
-          <t>Kjørt (UTC)</t>
+          <t>Skriptversjon</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" t="inlineStr">
+        <is>
+          <t>Kjørt (UTC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
         <is>
           <t>Dom fra finn_blaatt_hefte.py</t>
         </is>
@@ -1780,13 +1922,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D91"/>
+  <dimension ref="A1:D98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1819,17 +1961,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>hovedposter_kontroll</t>
+          <t>budsjettloep_merknad</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hovedposter</t>
+          <t>Budsjettløp</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>B13</t>
         </is>
       </c>
     </row>
@@ -1841,12 +1983,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>hovedposter_overskrift</t>
+          <t>budsjettloep_overskrift</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hovedposter</t>
+          <t>Budsjettløp</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1863,17 +2005,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>hovedposter_rnb_forslag</t>
+          <t>budsjettloep_start</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hovedposter</t>
+          <t>Budsjettløp</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>C24</t>
+          <t>B6</t>
         </is>
       </c>
     </row>
@@ -1885,7 +2027,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>hovedposter_rnb_nominell</t>
+          <t>hovedposter_kontroll</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1895,7 +2037,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>C25</t>
+          <t>D20</t>
         </is>
       </c>
     </row>
@@ -1907,7 +2049,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>hovedposter_rnb_realvekst</t>
+          <t>hovedposter_overskrift</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1917,7 +2059,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>C26</t>
+          <t>B5</t>
         </is>
       </c>
     </row>
@@ -1929,7 +2071,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>hovedposter_rnb_utgangspunkt</t>
+          <t>hovedposter_rnb_forslag</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1939,7 +2081,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>C23</t>
+          <t>C24</t>
         </is>
       </c>
     </row>
@@ -1951,7 +2093,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>hovedposter_start</t>
+          <t>hovedposter_rnb_nominell</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1961,7 +2103,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>B6</t>
+          <t>C25</t>
         </is>
       </c>
     </row>
@@ -1973,7 +2115,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>hovedposter_sum</t>
+          <t>hovedposter_rnb_realvekst</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1983,7 +2125,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>C26</t>
         </is>
       </c>
     </row>
@@ -1995,17 +2137,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>hovedtall_endring</t>
+          <t>hovedposter_rnb_utgangspunkt</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hovedtall</t>
+          <t>Hovedposter</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>C8</t>
+          <t>C23</t>
         </is>
       </c>
     </row>
@@ -2017,17 +2159,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>hovedtall_etikett_forslag</t>
+          <t>hovedposter_start</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Hovedtall</t>
+          <t>Hovedposter</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>B7</t>
+          <t>B6</t>
         </is>
       </c>
     </row>
@@ -2039,17 +2181,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>hovedtall_etikett_utgangspunkt</t>
+          <t>hovedposter_sum</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hovedtall</t>
+          <t>Hovedposter</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>B6</t>
+          <t>D19</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2203,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>hovedtall_forslag</t>
+          <t>hovedtall_endring</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2071,7 +2213,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C8</t>
         </is>
       </c>
     </row>
@@ -2083,7 +2225,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>hovedtall_nominell</t>
+          <t>hovedtall_etikett_forslag</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2093,7 +2235,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>C9</t>
+          <t>B7</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2247,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>hovedtall_prisavvik</t>
+          <t>hovedtall_etikett_utgangspunkt</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2115,7 +2257,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>B6</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2269,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>hovedtall_prisjustering</t>
+          <t>hovedtall_forslag</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2137,7 +2279,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>C15</t>
+          <t>C7</t>
         </is>
       </c>
     </row>
@@ -2149,7 +2291,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>hovedtall_prissats</t>
+          <t>hovedtall_nominell</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2159,7 +2301,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C9</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2313,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>hovedtall_realvekst_a</t>
+          <t>hovedtall_prisavvik</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2181,7 +2323,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>C19</t>
+          <t>C17</t>
         </is>
       </c>
     </row>
@@ -2193,7 +2335,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>hovedtall_realvekst_a_rnb</t>
+          <t>hovedtall_prisjustering</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2203,7 +2345,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C20</t>
+          <t>C15</t>
         </is>
       </c>
     </row>
@@ -2215,7 +2357,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>hovedtall_realvekst_b</t>
+          <t>hovedtall_prissats</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2225,7 +2367,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>C11</t>
+          <t>C10</t>
         </is>
       </c>
     </row>
@@ -2237,7 +2379,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>hovedtall_realvekst_b_rnb</t>
+          <t>hovedtall_realvekst_a</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2247,7 +2389,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>C12</t>
+          <t>C19</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2401,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>hovedtall_ren_sats</t>
+          <t>hovedtall_realvekst_a_rnb</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2269,7 +2411,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>C18</t>
+          <t>C20</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2423,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>hovedtall_rnb</t>
+          <t>hovedtall_realvekst_b</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2291,7 +2433,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>C21</t>
+          <t>C11</t>
         </is>
       </c>
     </row>
@@ -2303,7 +2445,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>hovedtall_sats_x_utgangspunkt</t>
+          <t>hovedtall_realvekst_b_rnb</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2313,7 +2455,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C12</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2467,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>hovedtall_utgangspunkt</t>
+          <t>hovedtall_ren_sats</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2335,7 +2477,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C18</t>
         </is>
       </c>
     </row>
@@ -2347,17 +2489,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>kilder_budsjettaar</t>
+          <t>hovedtall_rnb</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Kilder</t>
+          <t>Hovedtall</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C21</t>
         </is>
       </c>
     </row>
@@ -2369,17 +2511,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>kilder_content_length</t>
+          <t>hovedtall_sats_x_utgangspunkt</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Kilder</t>
+          <t>Hovedtall</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>C12</t>
+          <t>C16</t>
         </is>
       </c>
     </row>
@@ -2391,17 +2533,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>kilder_filnavn</t>
+          <t>hovedtall_utgangspunkt</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Kilder</t>
+          <t>Hovedtall</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C6</t>
         </is>
       </c>
     </row>
@@ -2413,7 +2555,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>kilder_finn_dom</t>
+          <t>kilder_budsjettaar</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2423,7 +2565,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>C33</t>
+          <t>C6</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2577,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>kilder_hentet</t>
+          <t>kilder_content_length</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2445,7 +2587,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>C12</t>
         </is>
       </c>
     </row>
@@ -2457,7 +2599,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>kilder_kjort</t>
+          <t>kilder_filnavn</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2467,7 +2609,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>C32</t>
+          <t>C10</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2621,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>kilder_kontroll_a</t>
+          <t>kilder_finn_dom</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2489,7 +2631,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>C27</t>
+          <t>C34</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2643,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>kilder_kontroll_b</t>
+          <t>kilder_hentet</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2511,7 +2653,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>C28</t>
+          <t>C13</t>
         </is>
       </c>
     </row>
@@ -2523,7 +2665,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>kilder_kontroll_c</t>
+          <t>kilder_kjort</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2533,7 +2675,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>C29</t>
+          <t>C33</t>
         </is>
       </c>
     </row>
@@ -2545,7 +2687,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>kilder_sha256</t>
+          <t>kilder_kontroll_a</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2555,7 +2697,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>C11</t>
+          <t>C28</t>
         </is>
       </c>
     </row>
@@ -2567,7 +2709,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>kilder_side_hovedtabell</t>
+          <t>kilder_kontroll_b</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2577,7 +2719,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C29</t>
         </is>
       </c>
     </row>
@@ -2589,7 +2731,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>kilder_side_institusjoner</t>
+          <t>kilder_kontroll_c</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2599,7 +2741,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>C23</t>
+          <t>C30</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2753,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>kilder_side_lukket</t>
+          <t>kilder_rnb</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2621,7 +2763,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>C22</t>
+          <t>C26</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2775,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>kilder_side_prisjustering</t>
+          <t>kilder_sha256</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2643,7 +2785,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>C19</t>
+          <t>C11</t>
         </is>
       </c>
     </row>
@@ -2655,7 +2797,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>kilder_side_resultat</t>
+          <t>kilder_side_hovedtabell</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2665,7 +2807,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>C20</t>
+          <t>C17</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2819,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>kilder_side_satser</t>
+          <t>kilder_side_institusjoner</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2687,7 +2829,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>C21</t>
+          <t>C23</t>
         </is>
       </c>
     </row>
@@ -2699,7 +2841,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>kilder_side_trykt</t>
+          <t>kilder_side_lukket</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2709,7 +2851,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>C18</t>
+          <t>C22</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2863,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>kilder_sider</t>
+          <t>kilder_side_prisjustering</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2731,7 +2873,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>C14</t>
+          <t>C19</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2885,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>kilder_sitat</t>
+          <t>kilder_side_resultat</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2753,7 +2895,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>C26</t>
+          <t>C20</t>
         </is>
       </c>
     </row>
@@ -2765,7 +2907,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>kilder_skript</t>
+          <t>kilder_side_satser</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2775,7 +2917,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>C30</t>
+          <t>C21</t>
         </is>
       </c>
     </row>
@@ -2787,7 +2929,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>kilder_skriptversjon</t>
+          <t>kilder_side_trykt</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2797,7 +2939,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>C31</t>
+          <t>C18</t>
         </is>
       </c>
     </row>
@@ -2809,7 +2951,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>kilder_tittel</t>
+          <t>kilder_sider</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2819,7 +2961,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>C8</t>
+          <t>C14</t>
         </is>
       </c>
     </row>
@@ -2831,7 +2973,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>kilder_url</t>
+          <t>kilder_sitat</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2841,7 +2983,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>C9</t>
+          <t>C27</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2995,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>kilder_utgave</t>
+          <t>kilder_skript</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2863,7 +3005,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C31</t>
         </is>
       </c>
     </row>
@@ -2875,17 +3017,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>resultat_merknad</t>
+          <t>kilder_skriptversjon</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Resultat</t>
+          <t>Kilder</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>B11</t>
+          <t>C32</t>
         </is>
       </c>
     </row>
@@ -2897,17 +3039,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>resultat_overskrift</t>
+          <t>kilder_tittel</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Resultat</t>
+          <t>Kilder</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>B5</t>
+          <t>C8</t>
         </is>
       </c>
     </row>
@@ -2919,17 +3061,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>resultat_start</t>
+          <t>kilder_url</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Resultat</t>
+          <t>Kilder</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>B6</t>
+          <t>C9</t>
         </is>
       </c>
     </row>
@@ -2941,17 +3083,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>satser_lukket_ramme_start</t>
+          <t>kilder_utgave</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Satser</t>
+          <t>Kilder</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>B32</t>
+          <t>C7</t>
         </is>
       </c>
     </row>
@@ -2963,17 +3105,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>satser_lukket_ramme_tomtekst</t>
+          <t>resultat_merknad</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Satser</t>
+          <t>Resultat</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>B32</t>
+          <t>B11</t>
         </is>
       </c>
     </row>
@@ -2985,17 +3127,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>satser_merknad</t>
+          <t>resultat_overskrift</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Satser</t>
+          <t>Resultat</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>B45</t>
+          <t>B5</t>
         </is>
       </c>
     </row>
@@ -3007,12 +3149,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>satser_open_ramme_start</t>
+          <t>resultat_start</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Satser</t>
+          <t>Resultat</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3029,7 +3171,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>satser_open_ramme_tomtekst</t>
+          <t>satser_lukket_ramme_start</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3039,7 +3181,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>B6</t>
+          <t>B32</t>
         </is>
       </c>
     </row>
@@ -3051,17 +3193,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>sektor_alle_overskrift</t>
+          <t>satser_lukket_ramme_tomtekst</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Sektor</t>
+          <t>Satser</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>B19</t>
+          <t>B32</t>
         </is>
       </c>
     </row>
@@ -3073,17 +3215,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>sektor_alle_start</t>
+          <t>satser_merknad</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Sektor</t>
+          <t>Satser</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>B20</t>
+          <t>B45</t>
         </is>
       </c>
     </row>
@@ -3095,12 +3237,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>sektor_universiteter_overskrift</t>
+          <t>satser_open_ramme_start</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Sektor</t>
+          <t>Satser</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3117,82 +3259,106 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>sektor_universiteter_start</t>
+          <t>satser_open_ramme_tomtekst</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Sektor</t>
+          <t>Satser</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>B7</t>
+          <t>B6</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>rad</t>
+          <t>celle</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>hovedposter_kontroll</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="n">
-        <v>20</v>
+          <t>sektor_alle_overskrift</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Sektor</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>B19</t>
+        </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>rad</t>
+          <t>celle</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>hovedposter_nest_siste</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="n">
-        <v>17</v>
+          <t>sektor_alle_start</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Sektor</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>B20</t>
+        </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>rad</t>
+          <t>celle</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>hovedposter_rnb_slutt</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="n">
-        <v>26</v>
+          <t>sektor_universiteter_overskrift</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Sektor</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>B6</t>
+        </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>rad</t>
+          <t>celle</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>hovedposter_rnb_start</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="n">
-        <v>23</v>
+          <t>sektor_universiteter_start</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Sektor</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>B7</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -3203,12 +3369,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>hovedposter_slutt</t>
+          <t>budsjettloep_nest_siste</t>
         </is>
       </c>
       <c r="C66" t="inlineStr"/>
       <c r="D66" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
     </row>
     <row r="67">
@@ -3219,12 +3385,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>hovedposter_start</t>
+          <t>budsjettloep_slutt</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="68">
@@ -3235,12 +3401,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>hovedposter_sum</t>
+          <t>budsjettloep_start</t>
         </is>
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
     <row r="69">
@@ -3251,12 +3417,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>hovedtall_hoveddel_slutt</t>
+          <t>hovedposter_kontroll</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="70">
@@ -3267,12 +3433,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>hovedtall_hoveddel_start</t>
+          <t>hovedposter_nest_siste</t>
         </is>
       </c>
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="71">
@@ -3283,12 +3449,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>hovedtall_kontroll_slutt</t>
+          <t>hovedposter_rnb_slutt</t>
         </is>
       </c>
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="72">
@@ -3299,12 +3465,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>hovedtall_kontroll_start</t>
+          <t>hovedposter_rnb_start</t>
         </is>
       </c>
       <c r="C72" t="inlineStr"/>
       <c r="D72" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="73">
@@ -3315,12 +3481,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>kilder_dokument_slutt</t>
+          <t>hovedposter_slutt</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
       <c r="D73" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="74">
@@ -3331,7 +3497,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>kilder_dokument_start</t>
+          <t>hovedposter_start</t>
         </is>
       </c>
       <c r="C74" t="inlineStr"/>
@@ -3347,12 +3513,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>kilder_kontroll_slutt</t>
+          <t>hovedposter_sum</t>
         </is>
       </c>
       <c r="C75" t="inlineStr"/>
       <c r="D75" t="n">
-        <v>33</v>
+        <v>19</v>
       </c>
     </row>
     <row r="76">
@@ -3363,12 +3529,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>kilder_kontroll_start</t>
+          <t>hovedtall_hoveddel_slutt</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
       <c r="D76" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
     </row>
     <row r="77">
@@ -3379,12 +3545,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>kilder_tabellsider_slutt</t>
+          <t>hovedtall_hoveddel_start</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>23</v>
+        <v>6</v>
       </c>
     </row>
     <row r="78">
@@ -3395,12 +3561,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>kilder_tabellsider_start</t>
+          <t>hovedtall_kontroll_slutt</t>
         </is>
       </c>
       <c r="C78" t="inlineStr"/>
       <c r="D78" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="79">
@@ -3411,12 +3577,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>resultat_nest_siste</t>
+          <t>hovedtall_kontroll_start</t>
         </is>
       </c>
       <c r="C79" t="inlineStr"/>
       <c r="D79" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="80">
@@ -3427,12 +3593,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>resultat_slutt</t>
+          <t>kilder_dokument_slutt</t>
         </is>
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="81">
@@ -3443,7 +3609,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>resultat_start</t>
+          <t>kilder_dokument_start</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
@@ -3459,12 +3625,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>satser_lukket_ramme_slutt</t>
+          <t>kilder_kontroll_slutt</t>
         </is>
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>43</v>
+        <v>34</v>
       </c>
     </row>
     <row r="83">
@@ -3475,12 +3641,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>satser_lukket_ramme_start</t>
+          <t>kilder_kontroll_start</t>
         </is>
       </c>
       <c r="C83" t="inlineStr"/>
       <c r="D83" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="84">
@@ -3491,12 +3657,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>satser_open_ramme_slutt</t>
+          <t>kilder_tabellsider_slutt</t>
         </is>
       </c>
       <c r="C84" t="inlineStr"/>
       <c r="D84" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="85">
@@ -3507,12 +3673,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>satser_open_ramme_start</t>
+          <t>kilder_tabellsider_start</t>
         </is>
       </c>
       <c r="C85" t="inlineStr"/>
       <c r="D85" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="86">
@@ -3523,12 +3689,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>sektor_alle_nest_siste</t>
+          <t>resultat_nest_siste</t>
         </is>
       </c>
       <c r="C86" t="inlineStr"/>
       <c r="D86" t="n">
-        <v>39</v>
+        <v>8</v>
       </c>
     </row>
     <row r="87">
@@ -3539,12 +3705,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>sektor_alle_slutt</t>
+          <t>resultat_slutt</t>
         </is>
       </c>
       <c r="C87" t="inlineStr"/>
       <c r="D87" t="n">
-        <v>40</v>
+        <v>9</v>
       </c>
     </row>
     <row r="88">
@@ -3555,12 +3721,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>sektor_alle_start</t>
+          <t>resultat_start</t>
         </is>
       </c>
       <c r="C88" t="inlineStr"/>
       <c r="D88" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="89">
@@ -3571,12 +3737,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>sektor_universiteter_nest_siste</t>
+          <t>satser_lukket_ramme_slutt</t>
         </is>
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>15</v>
+        <v>43</v>
       </c>
     </row>
     <row r="90">
@@ -3587,12 +3753,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>sektor_universiteter_slutt</t>
+          <t>satser_lukket_ramme_start</t>
         </is>
       </c>
       <c r="C90" t="inlineStr"/>
       <c r="D90" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
     </row>
     <row r="91">
@@ -3603,11 +3769,123 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>sektor_universiteter_start</t>
+          <t>satser_open_ramme_slutt</t>
         </is>
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>rad</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>satser_open_ramme_start</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>rad</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>sektor_alle_nest_siste</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>rad</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>sektor_alle_slutt</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>rad</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>sektor_alle_start</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>rad</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>sektor_universiteter_nest_siste</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>rad</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>sektor_universiteter_slutt</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>rad</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>sektor_universiteter_start</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="n">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
blatt-hefte: RNB review fixes (H1-H6, H8-H10)
RNB tillegg renamed endring (it can be negative); components carry post,
varig and the year a verifisert flag; 2023 marked unverified and shown
as such in Budsjettloep and the status prompt; 2025 basis (-1 091 in
vedtatt) recorded; tildelingsbrev ramme per year checked against the
vedtatt hefte in bygg_base. Runtime port: base vedtatt Y-1 must equal
the hefte utgangspunkt, else remark (rc 10). bygg_base refuses an empty
or shrinking base. Template labels no longer claim the RNB proposition
as source; realvekst labels name the RNB year; RNB regime derived from
the price-adjustment surplus, with an extra row for a durable RNB not
carried in the price column. Status prompt shows RNB effect in pp.
</commit_message>
<xml_diff>
--- a/skills/knowledge-management/blatt-hefte/assets/mal-rammeark.xlsx
+++ b/skills/knowledge-management/blatt-hefte/assets/mal-rammeark.xlsx
@@ -40,8 +40,10 @@
     <definedName name="hovedtall_realvekst_a_rnb">'Hovedtall'!$C$20</definedName>
     <definedName name="hovedtall_realvekst_b">'Hovedtall'!$C$11</definedName>
     <definedName name="hovedtall_realvekst_b_rnb">'Hovedtall'!$C$12</definedName>
+    <definedName name="hovedtall_realvekst_b_rnb_varig">'Hovedtall'!$C$21</definedName>
     <definedName name="hovedtall_ren_sats">'Hovedtall'!$C$18</definedName>
-    <definedName name="hovedtall_rnb">'Hovedtall'!$C$21</definedName>
+    <definedName name="hovedtall_rnb">'Hovedtall'!$C$23</definedName>
+    <definedName name="hovedtall_rnb_regime">'Hovedtall'!$C$22</definedName>
     <definedName name="hovedtall_sats_x_utgangspunkt">'Hovedtall'!$C$16</definedName>
     <definedName name="hovedtall_utgangspunkt">'Hovedtall'!$C$6</definedName>
     <definedName name="kilder_budsjettaar">'Kilder'!$C$6</definedName>
@@ -517,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C21"/>
+  <dimension ref="B2:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -612,11 +614,11 @@
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>Realvekst (metode b, med RNB)</t>
+          <t>Realvekst (metode b, med RNB &lt;år−1&gt; i utgangspunktet)</t>
         </is>
       </c>
       <c r="C12" s="5">
-        <f>IF('Hovedtall'!$C$21="","ikke oppgitt",('Hovedtall'!$C$8-'Hovedtall'!$C$15)/('Hovedtall'!$C$6+'Hovedtall'!$C$21))</f>
+        <f>IF('Hovedtall'!$C$23="","ikke oppgitt",('Hovedtall'!$C$8-'Hovedtall'!$C$15)/('Hovedtall'!$C$6+'Hovedtall'!$C$23))</f>
         <v/>
       </c>
     </row>
@@ -683,21 +685,39 @@
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>Realvekst (metode a, med RNB)</t>
+          <t>Realvekst (metode a, med RNB &lt;år−1&gt; i utgangspunktet)</t>
         </is>
       </c>
       <c r="C20" s="5">
-        <f>IF('Hovedtall'!$C$21="","ikke oppgitt",'Hovedtall'!$C$8/('Hovedtall'!$C$6+'Hovedtall'!$C$21)-'Hovedtall'!$C$10)</f>
+        <f>IF('Hovedtall'!$C$23="","ikke oppgitt",'Hovedtall'!$C$8/('Hovedtall'!$C$6+'Hovedtall'!$C$23)-'Hovedtall'!$C$10)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>Tillegg i RNB &lt;år-1&gt;, kap. 260 post 50, hentes fra RNB-proposisjonen; tom = ikke justert</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="n"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Realvekst (metode b) om RNB-endringen er varig og ikke inngår i prisjusteringskolonnen</t>
+        </is>
+      </c>
+      <c r="C21" s="5">
+        <f>IF('Hovedtall'!$C$23="","ikke oppgitt",('Hovedtall'!$C$7-('Hovedtall'!$C$6+'Hovedtall'!$C$23)-'Hovedtall'!$C$15)/('Hovedtall'!$C$6+'Hovedtall'!$C$23))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>RNB-regime (utledet av skriptet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>RNB-endring &lt;år−1&gt; for UiT, kap. 260 post 50, fra budsjettbasen (KDs supplerende tildelingsbrev); tom = ikke justert</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -754,12 +774,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>RNB-tillegg</t>
+          <t>RNB-endring, kap. 260 post 50</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Vedtatt inkl. RNB</t>
+          <t>Vedtatt etter RNB</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -825,7 +845,7 @@
     <row r="13">
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>RNB-tillegget er UiTs endring på kap. 260 post 50 i KDs supplerende tildelingsbrev nr. 1 etter revidert nasjonalbudsjett (juni/juli). Proposisjonen har bare sektortall, og blått hefte har ingen RNB-utgave. Realvekst «med RNB» i Hovedtall bruker RNB-tillegget for året før som del av utgangspunktet.</t>
+          <t>RNB-endringen er UiTs endring på kap. 260 post 50 i KDs supplerende tildelingsbrev nr. 1 etter revidert nasjonalbudsjett (juni/juli); den kan være negativ. Proposisjonen har bare sektortall, og blått hefte har ingen RNB-utgave. Hovedtall bruker RNB-endringen for året før som del av utgangspunktet. Kilder merket (uverifisert) er ikke kontrollert mot et offentlig dokument.</t>
         </is>
       </c>
     </row>
@@ -960,7 +980,7 @@
         </is>
       </c>
       <c r="C23" s="4">
-        <f>IF('Hovedtall'!$C$21="","ikke oppgitt",D6+'Hovedtall'!$C$21)</f>
+        <f>IF('Hovedtall'!$C$23="","ikke oppgitt",D6+'Hovedtall'!$C$23)</f>
         <v/>
       </c>
     </row>
@@ -971,7 +991,7 @@
         </is>
       </c>
       <c r="C24" s="4">
-        <f>IF('Hovedtall'!$C$21="","ikke oppgitt",D18+'Hovedtall'!$C$21)</f>
+        <f>IF('Hovedtall'!$C$23="","ikke oppgitt",D18+'Hovedtall'!$C$23)</f>
         <v/>
       </c>
     </row>
@@ -982,7 +1002,7 @@
         </is>
       </c>
       <c r="C25" s="5">
-        <f>IF('Hovedtall'!$C$21="","ikke oppgitt",(D18-D6)/(D6+'Hovedtall'!$C$21))</f>
+        <f>IF('Hovedtall'!$C$23="","ikke oppgitt",(D18-D6)/(D6+'Hovedtall'!$C$23))</f>
         <v/>
       </c>
     </row>
@@ -993,7 +1013,7 @@
         </is>
       </c>
       <c r="C26" s="5">
-        <f>IF('Hovedtall'!$C$21="","ikke oppgitt",(D18-D6-'Hovedtall'!$C$15)/(D6+'Hovedtall'!$C$21))</f>
+        <f>IF('Hovedtall'!$C$23="","ikke oppgitt",(D18-D6-'Hovedtall'!$C$15)/(D6+'Hovedtall'!$C$23))</f>
         <v/>
       </c>
     </row>
@@ -1928,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D98"/>
+  <dimension ref="A1:D100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2467,7 +2487,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>hovedtall_ren_sats</t>
+          <t>hovedtall_realvekst_b_rnb_varig</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2477,7 +2497,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>C18</t>
+          <t>C21</t>
         </is>
       </c>
     </row>
@@ -2489,7 +2509,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>hovedtall_rnb</t>
+          <t>hovedtall_ren_sats</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2499,7 +2519,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>C21</t>
+          <t>C18</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2531,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>hovedtall_sats_x_utgangspunkt</t>
+          <t>hovedtall_rnb</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2521,7 +2541,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C23</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2553,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>hovedtall_utgangspunkt</t>
+          <t>hovedtall_rnb_regime</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2543,7 +2563,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C22</t>
         </is>
       </c>
     </row>
@@ -2555,17 +2575,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>kilder_budsjettaar</t>
+          <t>hovedtall_sats_x_utgangspunkt</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Kilder</t>
+          <t>Hovedtall</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C16</t>
         </is>
       </c>
     </row>
@@ -2577,17 +2597,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>kilder_content_length</t>
+          <t>hovedtall_utgangspunkt</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Kilder</t>
+          <t>Hovedtall</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>C12</t>
+          <t>C6</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2619,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>kilder_filnavn</t>
+          <t>kilder_budsjettaar</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2609,7 +2629,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C6</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2641,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>kilder_finn_dom</t>
+          <t>kilder_content_length</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2631,7 +2651,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C12</t>
         </is>
       </c>
     </row>
@@ -2643,7 +2663,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>kilder_hentet</t>
+          <t>kilder_filnavn</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2653,7 +2673,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>C10</t>
         </is>
       </c>
     </row>
@@ -2665,7 +2685,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>kilder_kjort</t>
+          <t>kilder_finn_dom</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2675,7 +2695,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>C33</t>
+          <t>C34</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2707,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>kilder_kontroll_a</t>
+          <t>kilder_hentet</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2697,7 +2717,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>C28</t>
+          <t>C13</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2729,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>kilder_kontroll_b</t>
+          <t>kilder_kjort</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2719,7 +2739,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>C29</t>
+          <t>C33</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2751,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>kilder_kontroll_c</t>
+          <t>kilder_kontroll_a</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2741,7 +2761,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>C30</t>
+          <t>C28</t>
         </is>
       </c>
     </row>
@@ -2753,7 +2773,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>kilder_rnb</t>
+          <t>kilder_kontroll_b</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2763,7 +2783,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>C26</t>
+          <t>C29</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2795,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>kilder_sha256</t>
+          <t>kilder_kontroll_c</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2785,7 +2805,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>C11</t>
+          <t>C30</t>
         </is>
       </c>
     </row>
@@ -2797,7 +2817,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>kilder_side_hovedtabell</t>
+          <t>kilder_rnb</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2807,7 +2827,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C26</t>
         </is>
       </c>
     </row>
@@ -2819,7 +2839,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>kilder_side_institusjoner</t>
+          <t>kilder_sha256</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2829,7 +2849,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>C23</t>
+          <t>C11</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2861,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>kilder_side_lukket</t>
+          <t>kilder_side_hovedtabell</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2851,7 +2871,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>C22</t>
+          <t>C17</t>
         </is>
       </c>
     </row>
@@ -2863,7 +2883,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>kilder_side_prisjustering</t>
+          <t>kilder_side_institusjoner</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2873,7 +2893,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>C19</t>
+          <t>C23</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2905,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>kilder_side_resultat</t>
+          <t>kilder_side_lukket</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2895,7 +2915,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>C20</t>
+          <t>C22</t>
         </is>
       </c>
     </row>
@@ -2907,7 +2927,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>kilder_side_satser</t>
+          <t>kilder_side_prisjustering</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2917,7 +2937,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>C21</t>
+          <t>C19</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2949,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>kilder_side_trykt</t>
+          <t>kilder_side_resultat</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2939,7 +2959,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>C18</t>
+          <t>C20</t>
         </is>
       </c>
     </row>
@@ -2951,7 +2971,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>kilder_sider</t>
+          <t>kilder_side_satser</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2961,7 +2981,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>C14</t>
+          <t>C21</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2993,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>kilder_sitat</t>
+          <t>kilder_side_trykt</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2983,7 +3003,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>C27</t>
+          <t>C18</t>
         </is>
       </c>
     </row>
@@ -2995,7 +3015,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>kilder_skript</t>
+          <t>kilder_sider</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3005,7 +3025,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>C31</t>
+          <t>C14</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3037,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>kilder_skriptversjon</t>
+          <t>kilder_sitat</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3027,7 +3047,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>C32</t>
+          <t>C27</t>
         </is>
       </c>
     </row>
@@ -3039,7 +3059,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>kilder_tittel</t>
+          <t>kilder_skript</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3049,7 +3069,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>C8</t>
+          <t>C31</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3081,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>kilder_url</t>
+          <t>kilder_skriptversjon</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3071,7 +3091,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>C9</t>
+          <t>C32</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3103,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>kilder_utgave</t>
+          <t>kilder_tittel</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3093,7 +3113,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C8</t>
         </is>
       </c>
     </row>
@@ -3105,17 +3125,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>resultat_merknad</t>
+          <t>kilder_url</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Resultat</t>
+          <t>Kilder</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>B11</t>
+          <t>C9</t>
         </is>
       </c>
     </row>
@@ -3127,17 +3147,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>resultat_overskrift</t>
+          <t>kilder_utgave</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Resultat</t>
+          <t>Kilder</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>B5</t>
+          <t>C7</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3169,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>resultat_start</t>
+          <t>resultat_merknad</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3159,7 +3179,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>B6</t>
+          <t>B11</t>
         </is>
       </c>
     </row>
@@ -3171,17 +3191,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>satser_lukket_ramme_start</t>
+          <t>resultat_overskrift</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Satser</t>
+          <t>Resultat</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>B32</t>
+          <t>B5</t>
         </is>
       </c>
     </row>
@@ -3193,17 +3213,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>satser_lukket_ramme_tomtekst</t>
+          <t>resultat_start</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Satser</t>
+          <t>Resultat</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>B32</t>
+          <t>B6</t>
         </is>
       </c>
     </row>
@@ -3215,7 +3235,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>satser_merknad</t>
+          <t>satser_lukket_ramme_start</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3225,7 +3245,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>B45</t>
+          <t>B32</t>
         </is>
       </c>
     </row>
@@ -3237,7 +3257,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>satser_open_ramme_start</t>
+          <t>satser_lukket_ramme_tomtekst</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3247,7 +3267,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>B6</t>
+          <t>B32</t>
         </is>
       </c>
     </row>
@@ -3259,7 +3279,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>satser_open_ramme_tomtekst</t>
+          <t>satser_merknad</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3269,7 +3289,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>B6</t>
+          <t>B45</t>
         </is>
       </c>
     </row>
@@ -3281,17 +3301,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>sektor_alle_overskrift</t>
+          <t>satser_open_ramme_start</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Sektor</t>
+          <t>Satser</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>B19</t>
+          <t>B6</t>
         </is>
       </c>
     </row>
@@ -3303,17 +3323,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>sektor_alle_start</t>
+          <t>satser_open_ramme_tomtekst</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Sektor</t>
+          <t>Satser</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>B20</t>
+          <t>B6</t>
         </is>
       </c>
     </row>
@@ -3325,7 +3345,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>sektor_universiteter_overskrift</t>
+          <t>sektor_alle_overskrift</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3335,7 +3355,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>B6</t>
+          <t>B19</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3367,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>sektor_universiteter_start</t>
+          <t>sektor_alle_start</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3357,40 +3377,52 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>B7</t>
+          <t>B20</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>rad</t>
+          <t>celle</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>budsjettloep_nest_siste</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="n">
-        <v>10</v>
+          <t>sektor_universiteter_overskrift</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Sektor</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>B6</t>
+        </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>rad</t>
+          <t>celle</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>budsjettloep_slutt</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="n">
-        <v>11</v>
+          <t>sektor_universiteter_start</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Sektor</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>B7</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -3401,12 +3433,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>budsjettloep_start</t>
+          <t>budsjettloep_nest_siste</t>
         </is>
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="69">
@@ -3417,12 +3449,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>hovedposter_kontroll</t>
+          <t>budsjettloep_slutt</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="70">
@@ -3433,12 +3465,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>hovedposter_nest_siste</t>
+          <t>budsjettloep_start</t>
         </is>
       </c>
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
     </row>
     <row r="71">
@@ -3449,12 +3481,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>hovedposter_rnb_slutt</t>
+          <t>hovedposter_kontroll</t>
         </is>
       </c>
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="72">
@@ -3465,12 +3497,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>hovedposter_rnb_start</t>
+          <t>hovedposter_nest_siste</t>
         </is>
       </c>
       <c r="C72" t="inlineStr"/>
       <c r="D72" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="73">
@@ -3481,12 +3513,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>hovedposter_slutt</t>
+          <t>hovedposter_rnb_slutt</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
       <c r="D73" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="74">
@@ -3497,12 +3529,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>hovedposter_start</t>
+          <t>hovedposter_rnb_start</t>
         </is>
       </c>
       <c r="C74" t="inlineStr"/>
       <c r="D74" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
     </row>
     <row r="75">
@@ -3513,12 +3545,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>hovedposter_sum</t>
+          <t>hovedposter_slutt</t>
         </is>
       </c>
       <c r="C75" t="inlineStr"/>
       <c r="D75" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="76">
@@ -3529,12 +3561,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>hovedtall_hoveddel_slutt</t>
+          <t>hovedposter_start</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
       <c r="D76" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="77">
@@ -3545,12 +3577,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>hovedtall_hoveddel_start</t>
+          <t>hovedposter_sum</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
     </row>
     <row r="78">
@@ -3561,12 +3593,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>hovedtall_kontroll_slutt</t>
+          <t>hovedtall_hoveddel_slutt</t>
         </is>
       </c>
       <c r="C78" t="inlineStr"/>
       <c r="D78" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
     </row>
     <row r="79">
@@ -3577,12 +3609,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>hovedtall_kontroll_start</t>
+          <t>hovedtall_hoveddel_start</t>
         </is>
       </c>
       <c r="C79" t="inlineStr"/>
       <c r="D79" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="80">
@@ -3593,12 +3625,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>kilder_dokument_slutt</t>
+          <t>hovedtall_kontroll_slutt</t>
         </is>
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
     </row>
     <row r="81">
@@ -3609,12 +3641,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>kilder_dokument_start</t>
+          <t>hovedtall_kontroll_start</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
       <c r="D81" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="82">
@@ -3625,12 +3657,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>kilder_kontroll_slutt</t>
+          <t>kilder_dokument_slutt</t>
         </is>
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>34</v>
+        <v>14</v>
       </c>
     </row>
     <row r="83">
@@ -3641,12 +3673,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>kilder_kontroll_start</t>
+          <t>kilder_dokument_start</t>
         </is>
       </c>
       <c r="C83" t="inlineStr"/>
       <c r="D83" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
     </row>
     <row r="84">
@@ -3657,12 +3689,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>kilder_tabellsider_slutt</t>
+          <t>kilder_kontroll_slutt</t>
         </is>
       </c>
       <c r="C84" t="inlineStr"/>
       <c r="D84" t="n">
-        <v>23</v>
+        <v>34</v>
       </c>
     </row>
     <row r="85">
@@ -3673,12 +3705,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>kilder_tabellsider_start</t>
+          <t>kilder_kontroll_start</t>
         </is>
       </c>
       <c r="C85" t="inlineStr"/>
       <c r="D85" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
     </row>
     <row r="86">
@@ -3689,12 +3721,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>resultat_nest_siste</t>
+          <t>kilder_tabellsider_slutt</t>
         </is>
       </c>
       <c r="C86" t="inlineStr"/>
       <c r="D86" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="87">
@@ -3705,12 +3737,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>resultat_slutt</t>
+          <t>kilder_tabellsider_start</t>
         </is>
       </c>
       <c r="C87" t="inlineStr"/>
       <c r="D87" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="88">
@@ -3721,12 +3753,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>resultat_start</t>
+          <t>resultat_nest_siste</t>
         </is>
       </c>
       <c r="C88" t="inlineStr"/>
       <c r="D88" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="89">
@@ -3737,12 +3769,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>satser_lukket_ramme_slutt</t>
+          <t>resultat_slutt</t>
         </is>
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
     </row>
     <row r="90">
@@ -3753,12 +3785,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>satser_lukket_ramme_start</t>
+          <t>resultat_start</t>
         </is>
       </c>
       <c r="C90" t="inlineStr"/>
       <c r="D90" t="n">
-        <v>32</v>
+        <v>6</v>
       </c>
     </row>
     <row r="91">
@@ -3769,12 +3801,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>satser_open_ramme_slutt</t>
+          <t>satser_lukket_ramme_slutt</t>
         </is>
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>29</v>
+        <v>43</v>
       </c>
     </row>
     <row r="92">
@@ -3785,12 +3817,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>satser_open_ramme_start</t>
+          <t>satser_lukket_ramme_start</t>
         </is>
       </c>
       <c r="C92" t="inlineStr"/>
       <c r="D92" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
     </row>
     <row r="93">
@@ -3801,12 +3833,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>sektor_alle_nest_siste</t>
+          <t>satser_open_ramme_slutt</t>
         </is>
       </c>
       <c r="C93" t="inlineStr"/>
       <c r="D93" t="n">
-        <v>39</v>
+        <v>29</v>
       </c>
     </row>
     <row r="94">
@@ -3817,12 +3849,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>sektor_alle_slutt</t>
+          <t>satser_open_ramme_start</t>
         </is>
       </c>
       <c r="C94" t="inlineStr"/>
       <c r="D94" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
     </row>
     <row r="95">
@@ -3833,12 +3865,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>sektor_alle_start</t>
+          <t>sektor_alle_nest_siste</t>
         </is>
       </c>
       <c r="C95" t="inlineStr"/>
       <c r="D95" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
     </row>
     <row r="96">
@@ -3849,12 +3881,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>sektor_universiteter_nest_siste</t>
+          <t>sektor_alle_slutt</t>
         </is>
       </c>
       <c r="C96" t="inlineStr"/>
       <c r="D96" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
     </row>
     <row r="97">
@@ -3865,12 +3897,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>sektor_universiteter_slutt</t>
+          <t>sektor_alle_start</t>
         </is>
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="98">
@@ -3881,11 +3913,43 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>sektor_universiteter_start</t>
+          <t>sektor_universiteter_nest_siste</t>
         </is>
       </c>
       <c r="C98" t="inlineStr"/>
       <c r="D98" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>rad</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>sektor_universiteter_slutt</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>rad</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>sektor_universiteter_start</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="n">
         <v>7</v>
       </c>
     </row>

</xml_diff>